<commit_message>
docs(marketing): update Pro-first launch materials
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="223">
   <si>
     <t xml:space="preserve">HEYS · Маркетинг-методология</t>
   </si>
   <si>
-    <t xml:space="preserve">Сводная панель · снапшот 2026-06-09 · детали в файлах 01–13 и 05_Финмодель.xlsx</t>
+    <t xml:space="preserve">Сводная панель · снапшот 2026-06-10 · детали в файлах 01–22</t>
   </si>
   <si>
     <t xml:space="preserve">СУТЬ</t>
@@ -61,67 +61,52 @@
     <t xml:space="preserve">Удержание</t>
   </si>
   <si>
-    <t xml:space="preserve">Free</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 ₽</t>
+    <t xml:space="preserve">Self</t>
+  </si>
+  <si>
+    <t xml:space="preserve">490 ₽</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">лимит сканов</t>
-  </si>
-  <si>
-    <t xml:space="preserve">автопродление</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo / AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~990–1 490 ₽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">безлимит</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2 990–3 990 ₽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">раз/нед</t>
-  </si>
-  <si>
-    <t xml:space="preserve">куратор (ревью)</t>
+    <t xml:space="preserve">продление вручную</t>
   </si>
   <si>
     <t xml:space="preserve">Pro</t>
   </si>
   <si>
-    <t xml:space="preserve">~7 990 ₽*</t>
+    <t xml:space="preserve">7 990 ₽*</t>
   </si>
   <si>
     <t xml:space="preserve">ежедневно</t>
   </si>
   <si>
-    <t xml:space="preserve">2-я пара глаз</t>
-  </si>
-  <si>
-    <t xml:space="preserve">куратор</t>
+    <t xml:space="preserve">нет (ввод руками — фича)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">продление ведёт куратор</t>
   </si>
   <si>
     <t xml:space="preserve">Pro+</t>
   </si>
   <si>
-    <t xml:space="preserve">~14 990 ₽</t>
+    <t xml:space="preserve">14 990 ₽</t>
   </si>
   <si>
     <t xml:space="preserve">ежедн. +</t>
   </si>
   <si>
-    <t xml:space="preserve">*Ф0 (основатель), первые 15 фиксируются; в Ф1 ~9 900–10 900 ₽.  Удержание: без человека — автопродление; с куратором — продление ведёт куратор.</t>
+    <t xml:space="preserve">Solo / Lite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">архив</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R&amp;D / вопрос после Ф0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Ф0 (основатель), первые 8–12 фиксируются; в Ф1 ~9 900–10 900 ₽. Free — вход (квиз/демо/заявка), не тариф. Удержание: Self — вручную; Pro/Pro+ — продление ведёт куратор.</t>
   </si>
   <si>
     <t xml:space="preserve">ЭКОНОМИКА</t>
@@ -1119,16 +1104,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1260,14 +1245,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1276,7 +1253,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1288,7 +1265,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1745,48 +1722,48 @@
         <v>14</v>
       </c>
       <c r="E12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>16</v>
       </c>
       <c r="G12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
       <c r="B13" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="D13" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>14</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G14" s="2"/>
     </row>
@@ -1799,39 +1776,29 @@
         <v>25</v>
       </c>
       <c r="D15" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="14" t="s">
         <v>26</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>28</v>
       </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
-      <c r="B16" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>28</v>
-      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
       <c r="G16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
       <c r="B17" s="15" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
@@ -1846,7 +1813,7 @@
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="5" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -1857,37 +1824,37 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
       <c r="B20" s="16" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C20" s="16"/>
       <c r="D20" s="16" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E20" s="16"/>
       <c r="F20" s="17" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
       <c r="B21" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="19" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E21" s="19"/>
       <c r="F21" s="20" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
       <c r="B22" s="15" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
@@ -1902,7 +1869,7 @@
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
       <c r="B24" s="5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
@@ -1913,7 +1880,7 @@
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="21" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
@@ -1924,7 +1891,7 @@
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
       <c r="B26" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -1935,7 +1902,7 @@
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
       <c r="B27" s="21" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="21"/>
@@ -1946,7 +1913,7 @@
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
       <c r="B28" s="6" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -1961,7 +1928,7 @@
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
       <c r="B30" s="5" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -1972,7 +1939,7 @@
     <row r="31" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
       <c r="B31" s="6" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
@@ -1987,7 +1954,7 @@
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
       <c r="B33" s="5" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -1998,7 +1965,7 @@
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="2"/>
       <c r="B34" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
@@ -2013,7 +1980,7 @@
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
       <c r="B36" s="5" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -2024,7 +1991,7 @@
     <row r="37" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2"/>
       <c r="B37" s="6" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -2039,7 +2006,7 @@
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
       <c r="B39" s="5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -2050,7 +2017,7 @@
     <row r="40" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
       <c r="B40" s="22" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C40" s="22"/>
       <c r="D40" s="22"/>
@@ -2065,7 +2032,7 @@
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="2"/>
       <c r="B42" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
@@ -2076,7 +2043,7 @@
     <row r="43" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2"/>
       <c r="B43" s="23" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C43" s="23"/>
       <c r="D43" s="23"/>
@@ -2147,7 +2114,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -2157,7 +2124,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -2168,7 +2135,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -2178,7 +2145,7 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="27"/>
@@ -2204,7 +2171,7 @@
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2214,42 +2181,42 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="28" t="s">
         <v>61</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="28" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" s="31" t="s">
         <v>67</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="31" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2257,96 +2224,96 @@
         <v>8</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C14" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>90</v>
-      </c>
       <c r="F14" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F15" s="31" t="s">
         <v>14</v>
@@ -2354,88 +2321,88 @@
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="31" t="s">
         <v>96</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="D16" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="F16" s="31" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="29" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="31" t="s">
         <v>104</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" s="31" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="31" t="s">
         <v>110</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>112</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -2445,152 +2412,152 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B22" s="32" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C22" s="32"/>
       <c r="D22" s="32" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F22" s="32"/>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="29" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C23" s="31"/>
       <c r="D23" s="31" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F23" s="33"/>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="29" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C24" s="31"/>
       <c r="D24" s="31" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F24" s="33"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="29" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B25" s="31" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C25" s="31"/>
       <c r="D25" s="31" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E25" s="33" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F25" s="33"/>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="29" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B26" s="31" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C26" s="31"/>
       <c r="D26" s="31" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E26" s="33" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F26" s="33"/>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="29" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B27" s="31" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C27" s="31"/>
       <c r="D27" s="31" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F27" s="33"/>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="29" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B28" s="31" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C28" s="31"/>
       <c r="D28" s="31" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F28" s="33"/>
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="29" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B29" s="31" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C29" s="31"/>
       <c r="D29" s="31" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E29" s="33" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F29" s="33"/>
     </row>
     <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="29" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C30" s="31"/>
       <c r="D30" s="31" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E30" s="33" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F30" s="33"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="26" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B32" s="26"/>
       <c r="C32" s="26"/>
@@ -2600,7 +2567,7 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="27" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B33" s="27"/>
       <c r="C33" s="27"/>
@@ -2618,7 +2585,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="27" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B35" s="27"/>
       <c r="C35" s="27"/>
@@ -2636,7 +2603,7 @@
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="27" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
@@ -2654,7 +2621,7 @@
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="27" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B39" s="27"/>
       <c r="C39" s="27"/>
@@ -2672,7 +2639,7 @@
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="27" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B41" s="27"/>
       <c r="C41" s="27"/>
@@ -2690,7 +2657,7 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="26" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B43" s="26"/>
       <c r="C43" s="26"/>
@@ -2700,7 +2667,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="34" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B44" s="34"/>
       <c r="C44" s="34"/>
@@ -2769,361 +2736,361 @@
   <dimension ref="A1:G35"/>
   <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="35" width="2.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="35" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="35" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="35" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="2.5"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="36"/>
+      <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="36"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="36"/>
+      <c r="A2" s="2"/>
       <c r="B2" s="4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
-      <c r="G2" s="36"/>
+      <c r="G2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="36"/>
-      <c r="G3" s="36"/>
+      <c r="A3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="36"/>
+      <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="36"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36"/>
+      <c r="A5" s="2"/>
       <c r="B5" s="6" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="36"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36"/>
-      <c r="G6" s="36"/>
+      <c r="A6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36"/>
+      <c r="A7" s="2"/>
       <c r="B7" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="36"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36"/>
-      <c r="B8" s="37" t="s">
+      <c r="A8" s="2"/>
+      <c r="B8" s="35" t="s">
+        <v>159</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="F8" s="36"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2"/>
+      <c r="B9" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="39"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2"/>
+      <c r="B10" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="C8" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38" t="s">
+      <c r="C10" s="41" t="s">
         <v>165</v>
       </c>
-      <c r="F8" s="38"/>
-      <c r="G8" s="36"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36"/>
-      <c r="B9" s="39" t="s">
+      <c r="D10" s="41"/>
+      <c r="E10" s="42" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
+      <c r="B11" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41" t="s">
+      <c r="C11" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="F9" s="41"/>
-      <c r="G9" s="36"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="42" t="s">
+      <c r="D11" s="38"/>
+      <c r="E11" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="F11" s="39"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="40" t="s">
         <v>169</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C12" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="D10" s="43"/>
-      <c r="E10" s="44" t="s">
+      <c r="D12" s="41"/>
+      <c r="E12" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="F10" s="44"/>
-      <c r="G10" s="36"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36"/>
-      <c r="B11" s="39" t="s">
+      <c r="F12" s="42"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2"/>
+      <c r="B13" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C13" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="D11" s="40"/>
-      <c r="E11" s="41" t="s">
-        <v>168</v>
-      </c>
-      <c r="F11" s="41"/>
-      <c r="G11" s="36"/>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36"/>
-      <c r="B12" s="42" t="s">
+      <c r="D13" s="38"/>
+      <c r="E13" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="F13" s="39"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2"/>
+      <c r="B14" s="40" t="s">
         <v>174</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C14" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="D12" s="43"/>
-      <c r="E12" s="44" t="s">
+      <c r="D14" s="41"/>
+      <c r="E14" s="42" t="s">
+        <v>163</v>
+      </c>
+      <c r="F14" s="42"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="36"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="39" t="s">
-        <v>177</v>
-      </c>
-      <c r="C13" s="40" t="s">
-        <v>178</v>
-      </c>
-      <c r="D13" s="40"/>
-      <c r="E13" s="41" t="s">
-        <v>171</v>
-      </c>
-      <c r="F13" s="41"/>
-      <c r="G13" s="36"/>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="42" t="s">
-        <v>179</v>
-      </c>
-      <c r="C14" s="43" t="s">
-        <v>180</v>
-      </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="44" t="s">
-        <v>168</v>
-      </c>
-      <c r="F14" s="44"/>
-      <c r="G14" s="36"/>
-    </row>
-    <row r="15" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="G15" s="36"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="5" t="s">
-        <v>181</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="36"/>
+      <c r="G16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36"/>
+      <c r="A17" s="2"/>
       <c r="B17" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="36"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36"/>
-      <c r="G18" s="36"/>
+      <c r="A18" s="2"/>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36"/>
+      <c r="A19" s="2"/>
       <c r="B19" s="5" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="36"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
+      <c r="A20" s="2"/>
       <c r="B20" s="6" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="36"/>
+      <c r="G20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
+      <c r="A21" s="2"/>
       <c r="B21" s="21" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
-      <c r="G21" s="36"/>
+      <c r="G21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36"/>
+      <c r="A22" s="2"/>
       <c r="B22" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
-      <c r="G22" s="36"/>
+      <c r="G22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="G23" s="36"/>
+      <c r="A23" s="2"/>
+      <c r="G23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36"/>
+      <c r="A24" s="2"/>
       <c r="B24" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
-      <c r="G24" s="36"/>
+      <c r="G24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
+      <c r="A25" s="2"/>
       <c r="B25" s="6" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
-      <c r="G25" s="36"/>
+      <c r="G25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="36"/>
-      <c r="G26" s="36"/>
+      <c r="A26" s="2"/>
+      <c r="G26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36"/>
+      <c r="A27" s="2"/>
       <c r="B27" s="5" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
-      <c r="G27" s="36"/>
+      <c r="G27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="36"/>
+      <c r="A28" s="2"/>
       <c r="B28" s="6" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
-      <c r="G28" s="36"/>
+      <c r="G28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="36"/>
-      <c r="G29" s="36"/>
+      <c r="A29" s="2"/>
+      <c r="G29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="36"/>
+      <c r="A30" s="2"/>
       <c r="B30" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
-      <c r="G30" s="36"/>
+      <c r="G30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="36"/>
+      <c r="A31" s="2"/>
       <c r="B31" s="6" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
-      <c r="G31" s="36"/>
+      <c r="G31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="6.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="36"/>
-      <c r="G32" s="36"/>
+      <c r="A32" s="2"/>
+      <c r="G32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="36"/>
+      <c r="A33" s="2"/>
       <c r="B33" s="5" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
       <c r="F33" s="5"/>
-      <c r="G33" s="36"/>
+      <c r="G33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="36"/>
+      <c r="A34" s="2"/>
       <c r="B34" s="22" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C34" s="22"/>
       <c r="D34" s="22"/>
       <c r="E34" s="22"/>
       <c r="F34" s="22"/>
-      <c r="G34" s="36"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="36"/>
-      <c r="G35" s="36"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2"/>
+      <c r="G35" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="33">
@@ -3188,267 +3155,267 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="44"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="45" t="s">
+        <v>191</v>
+      </c>
+      <c r="B3" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>193</v>
+      </c>
+      <c r="E3" s="45" t="s">
+        <v>194</v>
+      </c>
+      <c r="F3" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="47" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="46" t="s">
         <v>196</v>
       </c>
-      <c r="B3" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="47" t="s">
+      <c r="B4" s="47" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="48" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="47" t="s">
-        <v>198</v>
-      </c>
-      <c r="E3" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="F3" s="47" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="48" t="s">
-        <v>201</v>
-      </c>
-      <c r="B4" s="49" t="n">
-        <v>15</v>
-      </c>
-      <c r="C4" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="D4" s="51"/>
-      <c r="E4" s="52" t="str">
+      <c r="D4" s="49"/>
+      <c r="E4" s="50" t="str">
         <f aca="false">IF(D4="","—",IF(D4&gt;=B4,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F4" s="53" t="s">
+      <c r="F4" s="51" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="B5" s="52"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="46" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" s="52"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="51" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="46" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="48" t="s">
-        <v>204</v>
-      </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="52" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="53" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="48" t="s">
-        <v>206</v>
-      </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="52" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="53" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="48" t="s">
-        <v>208</v>
-      </c>
-      <c r="B7" s="55" t="n">
+      <c r="B7" s="53" t="n">
         <v>0.4</v>
       </c>
-      <c r="C7" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="D7" s="56"/>
-      <c r="E7" s="52" t="str">
+      <c r="C7" s="48" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="54"/>
+      <c r="E7" s="50" t="str">
         <f aca="false">IF(D7="","—",IF(D7&gt;=B7,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F7" s="53" t="s">
-        <v>209</v>
+      <c r="F7" s="51" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="48" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="55" t="n">
+      <c r="A8" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="B8" s="53" t="n">
         <v>0.3</v>
       </c>
-      <c r="C8" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="D8" s="56"/>
-      <c r="E8" s="52" t="str">
+      <c r="C8" s="48" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="54"/>
+      <c r="E8" s="50" t="str">
         <f aca="false">IF(D8="","—",IF(D8&gt;=B8,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F8" s="53" t="s">
-        <v>211</v>
+      <c r="F8" s="51" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="48" t="s">
-        <v>212</v>
-      </c>
-      <c r="B9" s="57" t="n">
+      <c r="A9" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" s="55" t="n">
         <v>400</v>
       </c>
-      <c r="C9" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="58"/>
-      <c r="E9" s="52" t="str">
+      <c r="C9" s="48" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="56"/>
+      <c r="E9" s="50" t="str">
         <f aca="false">IF(D9="","—",IF(D9&lt;=B9,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F9" s="53" t="s">
-        <v>214</v>
+      <c r="F9" s="51" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="48" t="s">
-        <v>215</v>
-      </c>
-      <c r="B10" s="57" t="n">
+      <c r="A10" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" s="55" t="n">
         <v>10500</v>
       </c>
-      <c r="C10" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="D10" s="58"/>
-      <c r="E10" s="52" t="str">
+      <c r="C10" s="48" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="56"/>
+      <c r="E10" s="50" t="str">
         <f aca="false">IF(D10="","—",IF(D10&lt;=B10,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F10" s="53" t="s">
-        <v>216</v>
+      <c r="F10" s="51" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="48" t="s">
-        <v>217</v>
-      </c>
-      <c r="B11" s="59" t="n">
+      <c r="A11" s="46" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="D11" s="60"/>
-      <c r="E11" s="52" t="str">
+      <c r="C11" s="48" t="s">
+        <v>197</v>
+      </c>
+      <c r="D11" s="58"/>
+      <c r="E11" s="50" t="str">
         <f aca="false">IF(D11="","—",IF(D11&gt;=B11,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F11" s="53" t="s">
-        <v>218</v>
+      <c r="F11" s="51" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="48" t="s">
-        <v>219</v>
-      </c>
-      <c r="B12" s="55" t="n">
+      <c r="A12" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="B12" s="53" t="n">
         <v>0.09</v>
       </c>
-      <c r="C12" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="D12" s="56"/>
-      <c r="E12" s="52" t="str">
+      <c r="C12" s="48" t="s">
+        <v>208</v>
+      </c>
+      <c r="D12" s="54"/>
+      <c r="E12" s="50" t="str">
         <f aca="false">IF(D12="","—",IF(D12&lt;=B12,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F12" s="53" t="s">
-        <v>220</v>
+      <c r="F12" s="51" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="48" t="s">
-        <v>221</v>
-      </c>
-      <c r="B13" s="55" t="n">
+      <c r="A13" s="46" t="s">
+        <v>216</v>
+      </c>
+      <c r="B13" s="53" t="n">
         <v>0.05</v>
       </c>
-      <c r="C13" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="D13" s="56"/>
-      <c r="E13" s="52" t="str">
+      <c r="C13" s="48" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" s="54"/>
+      <c r="E13" s="50" t="str">
         <f aca="false">IF(D13="","—",IF(D13&lt;=B13,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F13" s="53" t="s">
-        <v>222</v>
+      <c r="F13" s="51" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="48" t="s">
-        <v>223</v>
-      </c>
-      <c r="B14" s="49" t="n">
+      <c r="A14" s="46" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="D14" s="51"/>
-      <c r="E14" s="52" t="str">
+      <c r="C14" s="48" t="s">
+        <v>197</v>
+      </c>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50" t="str">
         <f aca="false">IF(D14="","—",IF(D14&gt;=B14,"✅","⚠"))</f>
         <v>—</v>
       </c>
-      <c r="F14" s="53" t="s">
-        <v>224</v>
+      <c r="F14" s="51" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="48" t="s">
-        <v>225</v>
-      </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="52" t="s">
+      <c r="A15" s="46" t="s">
+        <v>220</v>
+      </c>
+      <c r="B15" s="52"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="53" t="s">
-        <v>226</v>
+      <c r="F15" s="51" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="46"/>
-      <c r="B16" s="46"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B17" s="25"/>
       <c r="C17" s="25"/>

</xml_diff>

<commit_message>
fix(marketing): sync pricing audit and legal versions
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -1634,7 +1634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="59" min="1" max="1"/>
@@ -2321,6 +2321,272 @@
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="60"/>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ГЛУБОКИЙ АУДИТ 2026-06-10 (детали — 29_Аудит_конкурентов_глубокий.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Слот «живой человек ЕЖЕДНЕВНО + персонально + КБЖУ-дневник» — ПУСТ глобально и в РФ. HEYS Pro 7 990 ₽ = треть Sekta-куратора, четверть частного нутрициолога.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>КАРТА «ЖИВОЙ ЧЕЛОВЕК» (приложения)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Игрок</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Человек</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Частота</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Цена/мес</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>РФ-оплата</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>HEYS Pro</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>куратор, персонально</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ежедневно 7/7</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>7 990 ₽</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Dietology.live</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>нутрициолог</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>заявлено ежедневно, без КБЖУ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>скрыта (~23–35К)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sekta (куратор)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>выпускник курсов</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>будни по графику, сб — нет</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>19 600–21 000 ₽</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Second Nature (UK)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>диетолог HCPC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>5/7, программа 12 нед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>~£33–40</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Noom</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>коуч «для галочки»</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>не ежедневно, шаблонно</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>~$17/мес год-экв</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Simple / трекеры / боты</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>нет (AI/—)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>200–1 300 ₽</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>частично</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ЦЕНОВАЯ ЛЕСТНИЦА РЫНКА, ₽/мес</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TG-боты 200–500 · трекеры RU 300–800 · западные 700–1 300 (оплата сломана) · марафоны 3 000–7 500 · Борменталь ~4 000+ (рассрочка) · Sekta 19 600–30 000 · частный нутрициолог 23 000–35 000. Вакуум 8–19К — наш Pro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ЛЕНДИНГИ: 5 ПАТТЕРНОВ ЛИДЕРОВ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1. Цифровой пруф над сгибом (рейтинг+масштаб+аватары) — у нас отзывы ниже сгиба.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2. Цена на главной скрыта почти у всех (кроме Sekta/марафонов) — наша открытая цена = отстройка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>3. Quiz-funnel — стандарт высокочековых (Simple/Noom/Sekta-тест).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>4. Кейсы «кг+срок+лицо»; наш канон без «-N кг» → нужны процессные кейсы (дни без срывов, % дневника).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>5. Вес пруфа растёт с чеком: инфлюенсеры → пресса → институции/наука (NHS, JAMA). Для 7 990 ₽ нужен тяжёлый пруф → медэксперт (27).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="32">
     <mergeCell ref="B25:C25"/>

</xml_diff>

<commit_message>
docs(marketing): focus release launch plan
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Конкуренты" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI-трекер" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Сводка" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Конкуренты" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Telegram" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="KPI-трекер" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2269,7 +2269,7 @@
     <row r="33" ht="30" customHeight="1" s="60">
       <c r="A33" s="86" t="inlineStr">
         <is>
-          <t>1. AI авто-распознавание = Solo-тариф — АРХИВ/R&amp;D после Ф0 (Pro-first, 19/21). В кураторском тарифе AI — «вторая пара глаз» (качество, не скорость); ввод остаётся ручным как фича. [R&amp;D после Ф0]</t>
+          <t>1. Пруф-инфраструктура для лендинга: реальные рейтинги/отзывы, лица специалистов, методология, научные ссылки, процессные кейсы. [РЕЛИЗ]</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
     <row r="35" ht="30" customHeight="1" s="60">
       <c r="A35" s="86" t="inlineStr">
         <is>
-          <t>2. Нативное приложение / RuStore — сторовые пруф-сигналы и доверие (закрыть PWA-разрыв). [NEXT]</t>
+          <t>2. SEO-калькуляторы после релиза: TDEE, BMI, дефицит, калории блюд — бесплатный верх воронки. [ПОСЛЕ РЕЛИЗА]</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
     <row r="37" ht="30" customHeight="1" s="60">
       <c r="A37" s="86" t="inlineStr">
         <is>
-          <t>3. Инфраструктура доказательств — счётчики, рейтинги, кейсы процесса, научные ссылки. [NEXT]</t>
+          <t>3. AI-ввод еды по фото / штрихкоду — отдельный R&amp;D после релиза; не обещание Pro-Ф0. [ПОСЛЕ РЕЛИЗА]</t>
         </is>
       </c>
     </row>
@@ -2293,17 +2293,13 @@
     <row r="39" ht="30" customHeight="1" s="60">
       <c r="A39" s="86" t="inlineStr">
         <is>
-          <t>4. SEO-калькуляторы (TDEE / калорийность / дефицит / BMI) — бесплатный органический трафик. [NEXT]</t>
+          <t>4. Нативное приложение / RuStore — сторовые рейтинги, бейджи и доверие; после первых данных. [ПОСЛЕ РЕЛИЗА]</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="60"/>
     <row r="41" ht="30" customHeight="1" s="60">
-      <c r="A41" s="86" t="inlineStr">
-        <is>
-          <t>5. Лендинг: поднять пруф выше + квантифицировать усилие + перевернуть стат «бросают без человека». [NOW]</t>
-        </is>
-      </c>
+      <c r="A41" s="86" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="60"/>
     <row r="43" ht="15.75" customHeight="1" s="60">
@@ -2322,266 +2318,266 @@
     </row>
     <row r="45" ht="15" customHeight="1" s="60"/>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="59" t="inlineStr">
         <is>
           <t>ГЛУБОКИЙ АУДИТ 2026-06-10 (детали — 29_Аудит_конкурентов_глубокий.md)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="59" t="inlineStr">
         <is>
           <t>Слот «живой человек ЕЖЕДНЕВНО + персонально + КБЖУ-дневник» — ПУСТ глобально и в РФ. HEYS Pro 7 990 ₽ = треть Sekta-куратора, четверть частного нутрициолога.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="59" t="inlineStr">
         <is>
           <t>КАРТА «ЖИВОЙ ЧЕЛОВЕК» (приложения)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="59" t="inlineStr">
         <is>
           <t>Игрок</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="59" t="inlineStr">
         <is>
           <t>Человек</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="59" t="inlineStr">
         <is>
           <t>Частота</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="59" t="inlineStr">
         <is>
           <t>Цена/мес</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="59" t="inlineStr">
         <is>
           <t>РФ-оплата</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="59" t="inlineStr">
         <is>
           <t>HEYS Pro</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="59" t="inlineStr">
         <is>
           <t>куратор, персонально</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="59" t="inlineStr">
         <is>
           <t>ежедневно 7/7</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="59" t="inlineStr">
         <is>
           <t>7 990 ₽</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="59" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="59" t="inlineStr">
         <is>
           <t>Dietology.live</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="59" t="inlineStr">
         <is>
           <t>нутрициолог</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="59" t="inlineStr">
         <is>
           <t>заявлено ежедневно, без КБЖУ</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="59" t="inlineStr">
         <is>
           <t>скрыта (~23–35К)</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="59" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="59" t="inlineStr">
         <is>
           <t>Sekta (куратор)</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="59" t="inlineStr">
         <is>
           <t>выпускник курсов</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="59" t="inlineStr">
         <is>
           <t>будни по графику, сб — нет</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="59" t="inlineStr">
         <is>
           <t>19 600–21 000 ₽</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="59" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="59" t="inlineStr">
         <is>
           <t>Second Nature (UK)</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="59" t="inlineStr">
         <is>
           <t>диетолог HCPC</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="59" t="inlineStr">
         <is>
           <t>5/7, программа 12 нед</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="59" t="inlineStr">
         <is>
           <t>~£33–40</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="59" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="59" t="inlineStr">
         <is>
           <t>Noom</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="59" t="inlineStr">
         <is>
           <t>коуч «для галочки»</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="59" t="inlineStr">
         <is>
           <t>не ежедневно, шаблонно</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="59" t="inlineStr">
         <is>
           <t>~$17/мес год-экв</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="59" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="59" t="inlineStr">
         <is>
           <t>Simple / трекеры / боты</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="59" t="inlineStr">
         <is>
           <t>нет (AI/—)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="59" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="59" t="inlineStr">
         <is>
           <t>200–1 300 ₽</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="59" t="inlineStr">
         <is>
           <t>частично</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="59" t="inlineStr">
         <is>
           <t>ЦЕНОВАЯ ЛЕСТНИЦА РЫНКА, ₽/мес</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="59" t="inlineStr">
         <is>
           <t>TG-боты 200–500 · трекеры RU 300–800 · западные 700–1 300 (оплата сломана) · марафоны 3 000–7 500 · Борменталь ~4 000+ (рассрочка) · Sekta 19 600–30 000 · частный нутрициолог 23 000–35 000. Вакуум 8–19К — наш Pro.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="59" t="inlineStr">
         <is>
           <t>ЛЕНДИНГИ: 5 ПАТТЕРНОВ ЛИДЕРОВ</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="59" t="inlineStr">
         <is>
           <t>1. Цифровой пруф над сгибом (рейтинг+масштаб+аватары) — у нас отзывы ниже сгиба.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="59" t="inlineStr">
         <is>
           <t>2. Цена на главной скрыта почти у всех (кроме Sekta/марафонов) — наша открытая цена = отстройка.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="59" t="inlineStr">
         <is>
           <t>3. Quiz-funnel — стандарт высокочековых (Simple/Noom/Sekta-тест).</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="59" t="inlineStr">
         <is>
           <t>4. Кейсы «кг+срок+лицо»; наш канон без «-N кг» → нужны процессные кейсы (дни без срывов, % дневника).</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="59" t="inlineStr">
         <is>
           <t>5. Вес пруфа растёт с чеком: инфлюенсеры → пресса → институции/наука (NHS, JAMA). Для 7 990 ₽ нужен тяжёлый пруф → медэксперт (27).</t>
         </is>

</xml_diff>

<commit_message>
docs(marketing): specify HEYS Start quiz funnel
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -1433,7 +1433,7 @@
       <c r="A26" s="61" t="n"/>
       <c r="B26" s="66" t="inlineStr">
         <is>
-          <t>2.  Бот «Твой тип срыва» (17) + контур измеримости (18): без них гейты roadmap 25 слепы.</t>
+          <t>HEYS Старт: бот «Твой тип срыва» (17) + контур измеримости (18). Алгоритм зафиксирован: 6 вопросов → сегмент → заявка на неделю; дальше BotFather, webhook и события quiz_start/quiz_complete/week_request.</t>
         </is>
       </c>
       <c r="G26" s="61" t="n"/>
@@ -2938,7 +2938,7 @@
       <c r="A25" s="61" t="n"/>
       <c r="B25" s="66" t="inlineStr">
         <is>
-          <t>Холодный (Ads/посев) и тёплый (контент) → бот-магнит (тест/чек-лист) → запись на неделю (по ёмкости куратора!) → куратор. Все ссылки — с UTM/промокодом (аналитика урезана под 152-ФЗ).</t>
+          <t>Холодный (Ads/посев) и тёплый (контент) → HEYS Старт: 6 вопросов «Твой тип срыва» → запись на неделю по ёмкости куратора → куратор. Все ссылки — с UTM/промокодом (аналитика урезана под 152-ФЗ).</t>
         </is>
       </c>
       <c r="G25" s="61" t="n"/>
@@ -2964,7 +2964,7 @@
       <c r="A28" s="61" t="n"/>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>ER ≥ 1,5–2%   ·   доля ботов в доноре &lt; 10%   ·   CPL под целевым   ·   лид→неделя ≥ 40%   ·   неделя→оплата ≥ 30%</t>
+          <t>ER ≥ 1,5–2%   ·   доля ботов в доноре &lt; 10%   ·   CPL под целевым   ·   quiz→неделя ≥ 40%   ·   неделя→оплата ≥ 30%</t>
         </is>
       </c>
       <c r="G28" s="61" t="n"/>

</xml_diff>

<commit_message>
docs(marketing): update roadmap, playbooks, PDn governance and ERID templates
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -1442,7 +1442,7 @@
       <c r="A27" s="61" t="n"/>
       <c r="B27" s="80" t="inlineStr">
         <is>
-          <t>3.  Юрист: договор НПД на результат (22 п.1.3); плейбук 23 вычитать вместе с договором.</t>
+          <t>Юрист/НПД не блокирует Ф0: договор внешнего куратора перенесён в 22 п.4.9 перед Ф1; сейчас фокус — ПДн/RKN gate и HEYS Старт.</t>
         </is>
       </c>
       <c r="G27" s="61" t="n"/>
@@ -1451,7 +1451,7 @@
       <c r="A28" s="61" t="n"/>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>4.  ERID — назначить ответственного (22 п.1.4) · запустить поиск медэксперта по RFP 27.</t>
+          <t>ERID закрыт: владелец назначен, регламент и шаблон посева — 33; дальше — поиск медэксперта по RFP 27.</t>
         </is>
       </c>
       <c r="G28" s="61" t="n"/>
@@ -2331,6 +2331,7 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="59" t="inlineStr">
         <is>
@@ -2527,6 +2528,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="59" t="inlineStr">
         <is>
@@ -2541,6 +2543,7 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="59" t="inlineStr">
         <is>
@@ -2990,7 +2993,7 @@
       <c r="A31" s="61" t="n"/>
       <c r="B31" s="66" t="inlineStr">
         <is>
-          <t>Свой контент в своём канале — ERID не нужен. Посевы/Ads — ERID + отчёт в ОРД до 30 числа + 3% рекламный сбор. Формулировки по COPY_VOICE.</t>
+          <t>Свой контент в своём канале — ERID не нужен. Посевы/Ads — ERID по регламенту 33: до публикации получить идентификатор, после показа отчитаться в ОРД до 30 календарных дней после месяца размещения. 3% сбор проверять договорно по роли площадки/исполнителя.</t>
         </is>
       </c>
       <c r="G31" s="61" t="n"/>

</xml_diff>

<commit_message>
chore(marketing): refresh launch dashboard
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -2678,7 +2678,7 @@
       <c r="A5" s="61" t="n"/>
       <c r="B5" s="66" t="inlineStr">
         <is>
-          <t>Ключевой канал для РФ-посевов и прогрева. Связка: канал (узнавание себя) → бот/карта срывов → заявка на неделю → куратор. Перед закупками проверять TGStat/Telemetr, считать CPL и заявки, не охваты.</t>
+          <t>Ключевой РФ-канал прогрева: узнавание себя → бот/карта срывов → заявка на неделю → куратор. Перед закупками: TGStat/Telemetr, UTM, целевой CPL 400 ₽ и позитивные соседние референсы, а не только фитнес/похудение.</t>
         </is>
       </c>
       <c r="G5" s="61" t="n"/>
@@ -2894,7 +2894,7 @@
       <c r="A20" s="61" t="n"/>
       <c r="B20" s="66" t="inlineStr">
         <is>
-          <t>Органика: полезный закреп после R0 → бот/карта срывов, тёплые репосты, взаимопиар с непрямыми каналами, реальные отзывы только с согласия.</t>
+          <t>Органика: контентный канал до R0 без сбора ПДн; после R0 — полезный закреп/бот, тёплые репосты, взаимопиар с непрямыми каналами и отзывы только с согласия. Закреп с оффером проверять как возможную саморекламу.</t>
         </is>
       </c>
       <c r="G20" s="61" t="n"/>
@@ -2903,7 +2903,7 @@
       <c r="A21" s="61" t="n"/>
       <c r="B21" s="80" t="inlineStr">
         <is>
-          <t>Посевы: только после TGStat/Telemetr-проверки — ER ≥ 1,5–2%, доля ботов &lt; 10%; тест с UTM/промокодом и замером заявок.</t>
+          <t>Посевы: не использовать TG-CH-001..007 как медиаплан. В тестовую выборку добавить бережное/осознанное питание, нутрициологов 30+, режим/выгорание; TGStat/Telemetr, ER доноров ≥1,5–2%, боты &lt;10%, UTM и замер заявок.</t>
         </is>
       </c>
       <c r="G21" s="61" t="n"/>
@@ -2912,7 +2912,7 @@
       <c r="A22" s="61" t="n"/>
       <c r="B22" s="66" t="inlineStr">
         <is>
-          <t>Telegram Ads: через eLama/реселлера условия перепроверять перед запуском; на июнь 2026 публично заявлены запуск с 0 € для юрлиц/ИП и комиссия 15% по акции. Планировать тест от CPL, вести на канал/магнит, не в оплату.</t>
+          <t>Telegram Ads: eLama/реселлер — условия перепроверять перед запуском. На июнь 2026 заявлены 0 € старт для юрлиц/ИП, оплата по факту; комиссия зависит от темы/бюджета и условий старта до 30.06.2026. Таргет — соседние архетипы, не похудательные каналы.</t>
         </is>
       </c>
       <c r="G22" s="61" t="n"/>
@@ -2938,7 +2938,7 @@
       <c r="A25" s="61" t="n"/>
       <c r="B25" s="66" t="inlineStr">
         <is>
-          <t>Холодный (Ads/посев) и тёплый (контент) → HEYS Старт: карта срывов / 6 вопросов → заявка на неделю по ёмкости куратора → куратор. Все ссылки — с UTM/промокодом; без сбора ПДн до R0.</t>
+          <t>Холодный/тёплый трафик → quiz_start → quiz_complete → week_request → trial_started → active_trial_d4 → payment. Не смешивать quiz→неделя, lead→trial_started и trial_started→payment; поток ограничен ёмкостью куратора.</t>
         </is>
       </c>
       <c r="G25" s="61" t="n"/>
@@ -2964,7 +2964,7 @@
       <c r="A28" s="61" t="n"/>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>ER ≥ 1,5–2% · доля ботов в доноре &lt; 10% · CPL под целевым · quiz→неделя ≥ 40% и неделя→оплата ≥ 30% как гипотезы до первых 30–50 лидов</t>
+          <t>CPL база ≤400 ₽ · lead→trial_started ≥40% · trial_started→payment ≥30% · quiz_complete→week_request отдельно · NPS триала · retention/отписки канала · first response time · SLA ≤5% · доля high-risk/RПП-risk лидов.</t>
         </is>
       </c>
       <c r="G28" s="61" t="n"/>
@@ -2990,7 +2990,7 @@
       <c r="A31" s="61" t="n"/>
       <c r="B31" s="66" t="inlineStr">
         <is>
-          <t>Свой контент в своём канале — ERID обычно не нужен. Посевы/Ads — ERID до публикации по регламенту 33, отчёт в ОРД не позднее 30 календарных дней после месяца размещения; 3% сбор проверять договорно по роли площадки/исполнителя.</t>
+          <t>Справочная органика без оффера обычно без ERID; закреп/баннер/пост саморекламы с CTA/ограниченными местами проверять по 33 и FAQ РКН, при сомнении заводить в ОРД. Посевы/Ads — ERID до публикации, договор, отчёт в ОРД.</t>
         </is>
       </c>
       <c r="G31" s="61" t="n"/>
@@ -3016,7 +3016,7 @@
       <c r="A34" s="61" t="n"/>
       <c r="B34" s="81" t="inlineStr">
         <is>
-          <t>Накрученные каналы; холодный трафик сразу в оплату; спам в чаты без разрешения; скидочный шум; «−N кг» / «24/7» / «психолог» / медицинские обещания.</t>
+          <t>Накрученные каналы; холодный трафик сразу в оплату; спам в чаты; скидочный шум; «−N кг» / «24/7» / «психолог» / медицинские обещания; публичные SLA «рядом каждый день» или «обычно час-два».</t>
         </is>
       </c>
       <c r="G34" s="61" t="n"/>
@@ -3073,7 +3073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="59" min="1" max="1"/>
@@ -3425,7 +3425,75 @@
       <c r="F16" s="105" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="60">
-      <c r="A17" s="84" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Отписки / retention канала</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>без резких отписок после CTA/посевов</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ниже лучше</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>First response time к заявке</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>по внутреннему SLA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ниже лучше</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NPS бесплатной недели</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>собирать после триала</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>выше лучше</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>High-risk / РПП-risk лиды</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>мониторить долю</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ниже лучше</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="84" t="inlineStr">
         <is>
           <t>✅ в норме · ⚠ ниже цели · — нет данных / нет числовой цели. Меняй цели под текущую фазу (Ф0/Ф1).</t>
         </is>

</xml_diff>

<commit_message>
docs(marketing): refresh pro positioning dashboard
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -1128,7 +1128,7 @@
       <c r="A5" s="61" t="n"/>
       <c r="B5" s="66" t="inlineStr">
         <is>
-          <t>Приложение + живой куратор + протоколы. Продаём заботу и анти-срыв — «вас ведут, а не оставляют с цифрами», а не диету.</t>
+          <t>Приложение + живой куратор + протоколы. Продаём внимательную внешнюю опору: вас ведут, держат контекст недели и помогают вернуться без стыда.</t>
         </is>
       </c>
       <c r="G5" s="61" t="n"/>
@@ -1154,7 +1154,7 @@
       <c r="A8" s="61" t="n"/>
       <c r="B8" s="66" t="inlineStr">
         <is>
-          <t>Между DIY-трекерами (нет человека, 0–500 ₽) и нутрициологом 1:1 (25 000+ ₽, нет приложения): ежедневный человек + приложение по доступной цене.</t>
+          <t>Между DIY-трекерами (нет человека, 0–500 ₽) и нутрициологом 1:1 (25 000+ ₽, нет приложения): куратор ведёт дневник + приложение по доступной цене.</t>
         </is>
       </c>
       <c r="G8" s="61" t="n"/>
@@ -2678,7 +2678,7 @@
       <c r="A5" s="61" t="n"/>
       <c r="B5" s="66" t="inlineStr">
         <is>
-          <t>Ключевой РФ-канал прогрева: узнавание себя → бот/карта срывов → заявка на неделю → куратор. Перед закупками: TGStat/Telemetr, UTM, целевой CPL 400 ₽ и позитивные соседние референсы, а не только фитнес/похудение.</t>
+          <t>Ключевой РФ-канал прогрева: узнавание себя → карта срывов/квиз → заявка на неделю → куратор как внимательная внешняя опора. Срывы — входная боль, продукт шире: дневник, контекст недели и мягкая ответственность. Перед закупками: TGStat/Telemetr, UTM, целевой CPL 400 ₽ и позитивные соседние референсы, а не только фитнес/похудение.</t>
         </is>
       </c>
       <c r="G5" s="61" t="n"/>
@@ -3425,68 +3425,58 @@
       <c r="F16" s="105" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="60">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="59" t="inlineStr">
         <is>
           <t>Отписки / retention канала</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>без резких отписок после CTA/посевов</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+    </row>
+    <row r="18">
+      <c r="A18" s="59" t="inlineStr">
+        <is>
+          <t>First response time к заявке</t>
+        </is>
+      </c>
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>по внутреннему SLA</t>
+        </is>
+      </c>
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>ниже лучше</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>First response time к заявке</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>по внутреннему SLA</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>ниже лучше</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="59" t="inlineStr">
         <is>
           <t>NPS бесплатной недели</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="59" t="inlineStr">
         <is>
           <t>собирать после триала</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="59" t="inlineStr">
         <is>
           <t>выше лучше</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="59" t="inlineStr">
         <is>
           <t>High-risk / РПП-risk лиды</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="59" t="inlineStr">
         <is>
           <t>мониторить долю</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="59" t="inlineStr">
         <is>
           <t>ниже лучше</t>
         </is>

</xml_diff>

<commit_message>
feat(platform): publish consolidated HEYS updates
</commit_message>
<xml_diff>
--- a/маркетинг/00_Сводная_панель.xlsx
+++ b/маркетинг/00_Сводная_панель.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" r:id="Rd279b15cf2b74531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Конкуренты" sheetId="2" r:id="R94afcbba21eb45bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram" sheetId="3" r:id="R67cb229499124d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI-трекер" sheetId="4" r:id="R49a0f67c68004ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" r:id="R66112785657f45e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Конкуренты" sheetId="2" r:id="Re8e2c16150854a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telegram" sheetId="3" r:id="R42bda12d258a4129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI-трекер" sheetId="4" r:id="Rdb99215f1c234953"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pro Спорт" sheetId="5" r:id="Rca2aa4b7fcc24f21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,12 +17,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="164" formatCode="0.0%"/>
     <x:numFmt numFmtId="165" formatCode="#,##0&quot; ₽&quot;;\(#,##0&quot; ₽)&quot;;\-"/>
     <x:numFmt numFmtId="166" formatCode="0.0\x"/>
+    <x:numFmt numFmtId="200" formatCode="#,##0 &quot;₽&quot;"/>
   </x:numFmts>
-  <x:fonts count="33">
+  <x:fonts count="37">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Arial"/>
@@ -197,8 +199,31 @@
       <x:color rgb="FF555555"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF607D8B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF263238"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2F8F83"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -270,8 +295,28 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153C4A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF22577A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="14">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -354,6 +399,41 @@
         <x:color rgb="FFD7E0E3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="hair">
+        <x:color rgb="FFC7D8D4"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D8D4"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -365,7 +445,7 @@
     <x:xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <x:xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="156">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
@@ -717,6 +797,114 @@
     </x:xf>
     <x:xf numFmtId="166" fontId="30" fillId="14" borderId="3" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="17" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="35" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="35" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -1151,30 +1339,20 @@
     </x:row>
     <x:row r="14" s="60" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="A14" s="61" t="n"/>
-      <x:c r="B14" s="69" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pro+</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14 990 ₽</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ежедн. +</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">нет (ввод руками — фича)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F14" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">продление ведёт куратор</x:t>
-        </x:is>
+      <x:c r="B14" s="69" t="str">
+        <x:v>Pro Спорт</x:v>
+      </x:c>
+      <x:c r="C14" s="70" t="str">
+        <x:v>19 990 ₽</x:v>
+      </x:c>
+      <x:c r="D14" s="70" t="str">
+        <x:v>один специалист: питание + тренировки</x:v>
+      </x:c>
+      <x:c r="E14" s="70" t="str">
+        <x:v>нет (ввод руками — фича)</x:v>
+      </x:c>
+      <x:c r="F14" s="70" t="str">
+        <x:v>ручное продление; 4 места</x:v>
       </x:c>
       <x:c r="G14" s="61" t="n"/>
     </x:row>
@@ -1218,10 +1396,8 @@
     </x:row>
     <x:row r="17" s="60" customFormat="1" ht="39" customHeight="1">
       <x:c r="A17" s="61" t="n"/>
-      <x:c r="B17" s="75" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">*Ф0 (основатель), первые 8–12 фиксируются; в Ф1 ~9 900–10 900 ₽. Free — вход (квиз/демо/заявка), не тариф. Удержание: Self — вручную; Pro/Pro+ — продление ведёт куратор.</x:t>
-        </x:is>
+      <x:c r="B17" s="75" t="str">
+        <x:v>* Pro — главный тариф и бесплатная неделя. Pro Спорт: пилот 4 места по 19 990 ₽; следующий набор 26 990 ₽ после ретроспективы.</x:v>
       </x:c>
       <x:c r="G17" s="61" t="n"/>
     </x:row>
@@ -1282,10 +1458,8 @@
     </x:row>
     <x:row r="22" s="60" customFormat="1" ht="39" customHeight="1">
       <x:c r="A22" s="61" t="n"/>
-      <x:c r="B22" s="75" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pro-first микс (Self 20/Pro 65/Pro+ 15): реальный CAC ~10 575 ₽ (триал = время куратора), базовый ~7 500 ₽. Реальный LTV:CAC 3,99× — выше цели. Кэш Ф0 при 15 клиентах ~111 000 ₽/мес. Пересчёт 2026-06-10 (05_Финмодель).</x:t>
-        </x:is>
+      <x:c r="B22" s="75" t="str">
+        <x:v>Pro-first: Self 490 / Pro 7 990 / Pro Спорт 19 990. Денежную экономику пилота не смешивать с нормализованной стоимостью замены основателя; подробности — 05, лист «Pro Спорт».</x:v>
       </x:c>
       <x:c r="G22" s="61" t="n"/>
     </x:row>
@@ -3355,4 +3529,276 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="153" t="str">
+        <x:v>Pro Спорт · решение пилота</x:v>
+      </x:c>
+      <x:c r="B1" s="153"/>
+      <x:c r="C1" s="153"/>
+      <x:c r="D1" s="153"/>
+      <x:c r="E1" s="153"/>
+      <x:c r="F1" s="153"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="126" t="str">
+        <x:v>Основатель совмещает куратора и специалиста по тренировкам; один общий контекст без передачи между людьми.</x:v>
+      </x:c>
+      <x:c r="B2" s="126"/>
+      <x:c r="C2" s="126"/>
+      <x:c r="D2" s="126"/>
+      <x:c r="E2" s="126"/>
+      <x:c r="F2" s="126"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="135" t="str">
+        <x:v>Параметр</x:v>
+      </x:c>
+      <x:c r="B4" s="136" t="str">
+        <x:v>Канон</x:v>
+      </x:c>
+      <x:c r="C4" s="154"/>
+      <x:c r="D4" s="154"/>
+      <x:c r="E4" s="154"/>
+      <x:c r="F4" s="154"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="142" t="str">
+        <x:v>Текущая цена</x:v>
+      </x:c>
+      <x:c r="B5" s="142" t="str">
+        <x:v>19 990 ₽/мес</x:v>
+      </x:c>
+      <x:c r="C5" s="154"/>
+      <x:c r="D5" s="154"/>
+      <x:c r="E5" s="154"/>
+      <x:c r="F5" s="154"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="142" t="str">
+        <x:v>Первый набор</x:v>
+      </x:c>
+      <x:c r="B6" s="142" t="str">
+        <x:v>4 принятых и оплативших клиента</x:v>
+      </x:c>
+      <x:c r="C6" s="154"/>
+      <x:c r="D6" s="154"/>
+      <x:c r="E6" s="154"/>
+      <x:c r="F6" s="154"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="142" t="str">
+        <x:v>Следующий набор</x:v>
+      </x:c>
+      <x:c r="B7" s="142" t="str">
+        <x:v>26 990 ₽/мес после ретроспективы</x:v>
+      </x:c>
+      <x:c r="C7" s="154"/>
+      <x:c r="D7" s="154"/>
+      <x:c r="E7" s="154"/>
+      <x:c r="F7" s="154"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="142" t="str">
+        <x:v>Главный тариф</x:v>
+      </x:c>
+      <x:c r="B8" s="142" t="str">
+        <x:v>Pro 7 990 ₽/мес</x:v>
+      </x:c>
+      <x:c r="C8" s="154"/>
+      <x:c r="D8" s="154"/>
+      <x:c r="E8" s="154"/>
+      <x:c r="F8" s="154"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="142" t="str">
+        <x:v>Бесплатная неделя</x:v>
+      </x:c>
+      <x:c r="B9" s="142" t="str">
+        <x:v>Только Pro</x:v>
+      </x:c>
+      <x:c r="C9" s="154"/>
+      <x:c r="D9" s="154"/>
+      <x:c r="E9" s="154"/>
+      <x:c r="F9" s="154"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="142" t="str">
+        <x:v>CTA Pro Спорт</x:v>
+      </x:c>
+      <x:c r="B10" s="142" t="str">
+        <x:v>Обсудить; без мгновенной покупки</x:v>
+      </x:c>
+      <x:c r="C10" s="154"/>
+      <x:c r="D10" s="154"/>
+      <x:c r="E10" s="154"/>
+      <x:c r="F10" s="154"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="142" t="str">
+        <x:v>Внутренние id</x:v>
+      </x:c>
+      <x:c r="B11" s="142" t="str">
+        <x:v>proPlus / proplus / pro_plus сохранены</x:v>
+      </x:c>
+      <x:c r="C11" s="154"/>
+      <x:c r="D11" s="154"/>
+      <x:c r="E11" s="154"/>
+      <x:c r="F11" s="154"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="143" t="str">
+        <x:v>Scale-gate</x:v>
+      </x:c>
+      <x:c r="B12" s="143" t="str">
+        <x:v>8 — после замера времени; 12 — только расчёт</x:v>
+      </x:c>
+      <x:c r="C12" s="154"/>
+      <x:c r="D12" s="154"/>
+      <x:c r="E12" s="154"/>
+      <x:c r="F12" s="154"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="154"/>
+      <x:c r="B13" s="154"/>
+      <x:c r="C13" s="154"/>
+      <x:c r="D13" s="154"/>
+      <x:c r="E13" s="154"/>
+      <x:c r="F13" s="154"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="155" t="str">
+        <x:v>ЭКОНОМИКА НА 1 КЛИЕНТА</x:v>
+      </x:c>
+      <x:c r="B14" s="155"/>
+      <x:c r="C14" s="155"/>
+      <x:c r="D14" s="155"/>
+      <x:c r="E14" s="155"/>
+      <x:c r="F14" s="155"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="135" t="str">
+        <x:v>Цена</x:v>
+      </x:c>
+      <x:c r="B15" s="150" t="str">
+        <x:v>Норм. прибыль</x:v>
+      </x:c>
+      <x:c r="C15" s="150" t="str">
+        <x:v>Норм. маржа</x:v>
+      </x:c>
+      <x:c r="D15" s="136" t="str">
+        <x:v>Первый месяц</x:v>
+      </x:c>
+      <x:c r="E15" s="154"/>
+      <x:c r="F15" s="154"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="151" t="n">
+        <x:v>14990</x:v>
+      </x:c>
+      <x:c r="B16" s="151" t="n">
+        <x:v>65.35</x:v>
+      </x:c>
+      <x:c r="C16" s="152" t="n">
+        <x:v>0.00436</x:v>
+      </x:c>
+      <x:c r="D16" s="151" t="n">
+        <x:v>-1434.65</x:v>
+      </x:c>
+      <x:c r="E16" s="154"/>
+      <x:c r="F16" s="154"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="151" t="n">
+        <x:v>19990</x:v>
+      </x:c>
+      <x:c r="B17" s="151" t="n">
+        <x:v>4890.35</x:v>
+      </x:c>
+      <x:c r="C17" s="152" t="n">
+        <x:v>0.24464</x:v>
+      </x:c>
+      <x:c r="D17" s="151" t="n">
+        <x:v>3390.35</x:v>
+      </x:c>
+      <x:c r="E17" s="154"/>
+      <x:c r="F17" s="154"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="151" t="n">
+        <x:v>26990</x:v>
+      </x:c>
+      <x:c r="B18" s="151" t="n">
+        <x:v>11645.35</x:v>
+      </x:c>
+      <x:c r="C18" s="152" t="n">
+        <x:v>0.43147</x:v>
+      </x:c>
+      <x:c r="D18" s="151" t="n">
+        <x:v>10145.35</x:v>
+      </x:c>
+      <x:c r="E18" s="154"/>
+      <x:c r="F18" s="154"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="142" t="str">
+        <x:v>Денежный пилот</x:v>
+      </x:c>
+      <x:c r="B19" s="142" t="str">
+        <x:v>Не включает оплату времени основателя</x:v>
+      </x:c>
+      <x:c r="C19" s="142" t="str">
+        <x:v>Время показывается отдельно</x:v>
+      </x:c>
+      <x:c r="D19" s="142" t="str">
+        <x:v>См. 05 / Pro Спорт</x:v>
+      </x:c>
+      <x:c r="E19" s="154"/>
+      <x:c r="F19" s="154"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="143" t="str">
+        <x:v>Capacity</x:v>
+      </x:c>
+      <x:c r="B20" s="143" t="str">
+        <x:v>4 клиента публично</x:v>
+      </x:c>
+      <x:c r="C20" s="143" t="str">
+        <x:v>8 после gate</x:v>
+      </x:c>
+      <x:c r="D20" s="143" t="str">
+        <x:v>12 расчётный предел</x:v>
+      </x:c>
+      <x:c r="E20" s="154"/>
+      <x:c r="F20" s="154"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A14:F14"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>